<commit_message>
fix: style the template
</commit_message>
<xml_diff>
--- a/server/template.xlsx
+++ b/server/template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30610"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gianmario.tartaglion\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC2BC9DD-DE08-4F81-8FD3-39CD3B3888BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B102234-36D6-41E2-9032-EE30D086D4F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{CA9CAA66-B28B-4A23-B6A6-87BF683D5A9F}"/>
   </bookViews>
@@ -479,8 +479,8 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
+    <col min="1" max="1" width="33.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
     <col min="3" max="3" width="60.5703125" customWidth="1"/>
     <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.140625" bestFit="1" customWidth="1"/>
@@ -489,7 +489,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">

</xml_diff>